<commit_message>
Put Yuri last in the Master roster, and import his KPI targets
Two mistakes in the first pass.

He was first in the list, which pushed every other rep down a row on
every dashboard and roster. Appending him leaves existing positions
where people expect them.

And he was missing has_kpi, so Master would not have imported his
targets tab - his KPI columns would have sat blank while his book
filled up, which reads as a broken sheet rather than a missing flag.
</commit_message>
<xml_diff>
--- a/Daily_Gamba_Master_Dashboard_v24.xlsx
+++ b/Daily_Gamba_Master_Dashboard_v24.xlsx
@@ -14,71 +14,71 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overdue Follow-Ups" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team &amp; KPI Targets" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri Book" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri ActivityLog" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri VIPTeam" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri FtdList" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri KPI" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna Book" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna ActivityLog" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna VIPTeam" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna FtdList" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna KPI" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat Book" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat ActivityLog" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat VIPTeam" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat FtdList" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat KPI" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella Book" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella ActivityLog" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella VIPTeam" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella FtdList" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella KPI" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist Book" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist ActivityLog" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist VIPTeam" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist FtdList" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist KPI" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb Book" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb ActivityLog" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb VIPTeam" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb FtdList" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb KPI" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey Book" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey ActivityLog" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey VIPTeam" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey FtdList" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey KPI" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok Book" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok ActivityLog" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok VIPTeam" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok FtdList" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok KPI" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen Book" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen ActivityLog" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen VIPTeam" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen FtdList" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen KPI" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko Book" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko ActivityLog" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko VIPTeam" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko FtdList" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko KPI" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept Book" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept ActivityLog" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept VIPTeam" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept FtdList" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept KPI" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily Book" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily ActivityLog" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily VIPTeam" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily FtdList" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily KPI" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime Book" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime ActivityLog" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime VIPTeam" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime FtdList" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime KPI" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna Book" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna ActivityLog" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna VIPTeam" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna FtdList" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Tuna KPI" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat Book" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat ActivityLog" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat VIPTeam" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat FtdList" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Plat KPI" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella Book" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella ActivityLog" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella VIPTeam" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella FtdList" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Chella KPI" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist Book" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist ActivityLog" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist VIPTeam" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist FtdList" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Moneyheist KPI" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb Book" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb ActivityLog" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb VIPTeam" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb FtdList" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seb KPI" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey Book" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey ActivityLog" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey VIPTeam" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey FtdList" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Pricey KPI" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok Book" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok ActivityLog" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok VIPTeam" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok FtdList" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Seanok KPI" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen Book" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen ActivityLog" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen VIPTeam" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen FtdList" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Gwen KPI" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko Book" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko ActivityLog" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko VIPTeam" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko FtdList" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Miko KPI" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept Book" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept ActivityLog" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept VIPTeam" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept FtdList" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Concept KPI" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily Book" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily ActivityLog" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily VIPTeam" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily FtdList" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Daily KPI" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime Book" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime ActivityLog" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime VIPTeam" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime FtdList" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Prime KPI" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri Book" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri ActivityLog" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri VIPTeam" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri FtdList" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Import Yuri KPI" sheetId="72" state="visible" r:id="rId72"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Player DB'!$A$4:$P$2604</definedName>
@@ -788,7 +788,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!B4:B203"),IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!AC4:AC203"),IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!W4:W203"),IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!B4:B203"),IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!AC4:AC203"),IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!W4:W203"),IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -808,7 +808,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -828,7 +828,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -848,7 +848,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -868,7 +868,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -888,7 +888,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!B4:B203"),IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!AC4:AC203"),IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!W4:W203"),IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!B4:B203"),IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!AC4:AC203"),IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!W4:W203"),IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -908,7 +908,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -928,7 +928,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -948,7 +948,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -968,7 +968,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <f>IFERROR(FILTER({IF('_Import Yuri Book'!B1:B200="","","Yuri"), '_Import Yuri Book'!A1:F200, '_Import Yuri Book'!H1:O200, IFERROR('_Import Yuri VIPTeam'!B1:B200,""); IF('_Import Tuna Book'!B1:B200="","","Tuna"), '_Import Tuna Book'!A1:F200, '_Import Tuna Book'!H1:O200, IFERROR('_Import Tuna VIPTeam'!B1:B200,""); IF('_Import Plat Book'!B1:B200="","","Plat"), '_Import Plat Book'!A1:F200, '_Import Plat Book'!H1:O200, IFERROR('_Import Plat VIPTeam'!B1:B200,""); IF('_Import Chella Book'!B1:B200="","","Chella"), '_Import Chella Book'!A1:F200, '_Import Chella Book'!H1:O200, IFERROR('_Import Chella VIPTeam'!B1:B200,""); IF('_Import Moneyheist Book'!B1:B200="","","Moneyheist"), '_Import Moneyheist Book'!A1:F200, '_Import Moneyheist Book'!H1:O200, IFERROR('_Import Moneyheist VIPTeam'!B1:B200,""); IF('_Import Seb Book'!B1:B200="","","Seb"), '_Import Seb Book'!A1:F200, '_Import Seb Book'!H1:O200, IFERROR('_Import Seb VIPTeam'!B1:B200,""); IF('_Import Pricey Book'!B1:B200="","","Pricey"), '_Import Pricey Book'!A1:F200, '_Import Pricey Book'!H1:O200, IFERROR('_Import Pricey VIPTeam'!B1:B200,""); IF('_Import Seanok Book'!B1:B200="","","Seanok"), '_Import Seanok Book'!A1:F200, '_Import Seanok Book'!H1:O200, IFERROR('_Import Seanok VIPTeam'!B1:B200,""); IF('_Import Gwen Book'!B1:B200="","","Gwen"), '_Import Gwen Book'!A1:F200, '_Import Gwen Book'!H1:O200, IFERROR('_Import Gwen VIPTeam'!B1:B200,""); IF('_Import Miko Book'!B1:B200="","","Miko"), '_Import Miko Book'!A1:F200, '_Import Miko Book'!H1:O200, IFERROR('_Import Miko VIPTeam'!B1:B200,""); IF('_Import Concept Book'!B1:B200="","","Concept"), '_Import Concept Book'!A1:F200, '_Import Concept Book'!H1:O200, IFERROR('_Import Concept VIPTeam'!B1:B200,""); IF('_Import Daily Book'!B1:B200="","","Daily"), '_Import Daily Book'!A1:F200, '_Import Daily Book'!H1:O200, IFERROR('_Import Daily VIPTeam'!B1:B200,""); IF('_Import Prime Book'!B1:B200="","","Prime"), '_Import Prime Book'!A1:F200, '_Import Prime Book'!H1:O200, IFERROR('_Import Prime VIPTeam'!B1:B200,"")}, {'_Import Yuri Book'!B1:B200&lt;&gt;""; '_Import Tuna Book'!B1:B200&lt;&gt;""; '_Import Plat Book'!B1:B200&lt;&gt;""; '_Import Chella Book'!B1:B200&lt;&gt;""; '_Import Moneyheist Book'!B1:B200&lt;&gt;""; '_Import Seb Book'!B1:B200&lt;&gt;""; '_Import Pricey Book'!B1:B200&lt;&gt;""; '_Import Seanok Book'!B1:B200&lt;&gt;""; '_Import Gwen Book'!B1:B200&lt;&gt;""; '_Import Miko Book'!B1:B200&lt;&gt;""; '_Import Concept Book'!B1:B200&lt;&gt;""; '_Import Daily Book'!B1:B200&lt;&gt;""; '_Import Prime Book'!B1:B200&lt;&gt;""}), "")</f>
+        <f>IFERROR(FILTER({IF('_Import Tuna Book'!B1:B200="","","Tuna"), '_Import Tuna Book'!A1:F200, '_Import Tuna Book'!H1:O200, IFERROR('_Import Tuna VIPTeam'!B1:B200,""); IF('_Import Plat Book'!B1:B200="","","Plat"), '_Import Plat Book'!A1:F200, '_Import Plat Book'!H1:O200, IFERROR('_Import Plat VIPTeam'!B1:B200,""); IF('_Import Chella Book'!B1:B200="","","Chella"), '_Import Chella Book'!A1:F200, '_Import Chella Book'!H1:O200, IFERROR('_Import Chella VIPTeam'!B1:B200,""); IF('_Import Moneyheist Book'!B1:B200="","","Moneyheist"), '_Import Moneyheist Book'!A1:F200, '_Import Moneyheist Book'!H1:O200, IFERROR('_Import Moneyheist VIPTeam'!B1:B200,""); IF('_Import Seb Book'!B1:B200="","","Seb"), '_Import Seb Book'!A1:F200, '_Import Seb Book'!H1:O200, IFERROR('_Import Seb VIPTeam'!B1:B200,""); IF('_Import Pricey Book'!B1:B200="","","Pricey"), '_Import Pricey Book'!A1:F200, '_Import Pricey Book'!H1:O200, IFERROR('_Import Pricey VIPTeam'!B1:B200,""); IF('_Import Seanok Book'!B1:B200="","","Seanok"), '_Import Seanok Book'!A1:F200, '_Import Seanok Book'!H1:O200, IFERROR('_Import Seanok VIPTeam'!B1:B200,""); IF('_Import Gwen Book'!B1:B200="","","Gwen"), '_Import Gwen Book'!A1:F200, '_Import Gwen Book'!H1:O200, IFERROR('_Import Gwen VIPTeam'!B1:B200,""); IF('_Import Miko Book'!B1:B200="","","Miko"), '_Import Miko Book'!A1:F200, '_Import Miko Book'!H1:O200, IFERROR('_Import Miko VIPTeam'!B1:B200,""); IF('_Import Concept Book'!B1:B200="","","Concept"), '_Import Concept Book'!A1:F200, '_Import Concept Book'!H1:O200, IFERROR('_Import Concept VIPTeam'!B1:B200,""); IF('_Import Daily Book'!B1:B200="","","Daily"), '_Import Daily Book'!A1:F200, '_Import Daily Book'!H1:O200, IFERROR('_Import Daily VIPTeam'!B1:B200,""); IF('_Import Prime Book'!B1:B200="","","Prime"), '_Import Prime Book'!A1:F200, '_Import Prime Book'!H1:O200, IFERROR('_Import Prime VIPTeam'!B1:B200,""); IF('_Import Yuri Book'!B1:B200="","","Yuri"), '_Import Yuri Book'!A1:F200, '_Import Yuri Book'!H1:O200, IFERROR('_Import Yuri VIPTeam'!B1:B200,"")}, {'_Import Tuna Book'!B1:B200&lt;&gt;""; '_Import Plat Book'!B1:B200&lt;&gt;""; '_Import Chella Book'!B1:B200&lt;&gt;""; '_Import Moneyheist Book'!B1:B200&lt;&gt;""; '_Import Seb Book'!B1:B200&lt;&gt;""; '_Import Pricey Book'!B1:B200&lt;&gt;""; '_Import Seanok Book'!B1:B200&lt;&gt;""; '_Import Gwen Book'!B1:B200&lt;&gt;""; '_Import Miko Book'!B1:B200&lt;&gt;""; '_Import Concept Book'!B1:B200&lt;&gt;""; '_Import Daily Book'!B1:B200&lt;&gt;""; '_Import Prime Book'!B1:B200&lt;&gt;""; '_Import Yuri Book'!B1:B200&lt;&gt;""}), "")</f>
         <v/>
       </c>
       <c r="H5" s="8" t="n"/>
@@ -16736,7 +16736,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!B4:B203"),IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!AC4:AC203"),IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!W4:W203"),IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!B4:B203"),IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!AC4:AC203"),IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!W4:W203"),IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -16756,7 +16756,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Plat - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -16776,7 +16776,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1Fk54o-UXm0eMEzi-5e1_yqmrFmyLaoRfMjLThRQRKoY", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -16796,7 +16796,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -16816,7 +16816,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -16836,7 +16836,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!B4:B203"),IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!AC4:AC203"),IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!W4:W203"),IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!B4:B203"),IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!AC4:AC203"),IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!W4:W203"),IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -16856,7 +16856,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Chella - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -16876,7 +16876,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1RQVsxe270nT9Dw9GCvmcwlzuVL6D3QFNCmm1KpZOGp4", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -16896,7 +16896,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -16916,7 +16916,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -16995,7 +16995,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <f>IFERROR(FILTER({IFERROR(IF('_Import Yuri FtdList'!A1:A200="","","Yuri"),""), IFERROR('_Import Yuri FtdList'!A1:D200,""); IFERROR(IF('_Import Tuna FtdList'!A1:A200="","","Tuna"),""), IFERROR('_Import Tuna FtdList'!A1:D200,""); IFERROR(IF('_Import Plat FtdList'!A1:A200="","","Plat"),""), IFERROR('_Import Plat FtdList'!A1:D200,""); IFERROR(IF('_Import Chella FtdList'!A1:A200="","","Chella"),""), IFERROR('_Import Chella FtdList'!A1:D200,""); IFERROR(IF('_Import Moneyheist FtdList'!A1:A200="","","Moneyheist"),""), IFERROR('_Import Moneyheist FtdList'!A1:D200,""); IFERROR(IF('_Import Seb FtdList'!A1:A200="","","Seb"),""), IFERROR('_Import Seb FtdList'!A1:D200,""); IFERROR(IF('_Import Pricey FtdList'!A1:A200="","","Pricey"),""), IFERROR('_Import Pricey FtdList'!A1:D200,""); IFERROR(IF('_Import Seanok FtdList'!A1:A200="","","Seanok"),""), IFERROR('_Import Seanok FtdList'!A1:D200,""); IFERROR(IF('_Import Gwen FtdList'!A1:A200="","","Gwen"),""), IFERROR('_Import Gwen FtdList'!A1:D200,""); IFERROR(IF('_Import Miko FtdList'!A1:A200="","","Miko"),""), IFERROR('_Import Miko FtdList'!A1:D200,""); IFERROR(IF('_Import Concept FtdList'!A1:A200="","","Concept"),""), IFERROR('_Import Concept FtdList'!A1:D200,""); IFERROR(IF('_Import Daily FtdList'!A1:A200="","","Daily"),""), IFERROR('_Import Daily FtdList'!A1:D200,""); IFERROR(IF('_Import Prime FtdList'!A1:A200="","","Prime"),""), IFERROR('_Import Prime FtdList'!A1:D200,"")}, {IFERROR('_Import Yuri FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Tuna FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Plat FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Chella FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Moneyheist FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Seb FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Pricey FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Seanok FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Gwen FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Miko FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Concept FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Daily FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Prime FtdList'!A1:A200&lt;&gt;"",FALSE)}), "")</f>
+        <f>IFERROR(FILTER({IFERROR(IF('_Import Tuna FtdList'!A1:A200="","","Tuna"),""), IFERROR('_Import Tuna FtdList'!A1:D200,""); IFERROR(IF('_Import Plat FtdList'!A1:A200="","","Plat"),""), IFERROR('_Import Plat FtdList'!A1:D200,""); IFERROR(IF('_Import Chella FtdList'!A1:A200="","","Chella"),""), IFERROR('_Import Chella FtdList'!A1:D200,""); IFERROR(IF('_Import Moneyheist FtdList'!A1:A200="","","Moneyheist"),""), IFERROR('_Import Moneyheist FtdList'!A1:D200,""); IFERROR(IF('_Import Seb FtdList'!A1:A200="","","Seb"),""), IFERROR('_Import Seb FtdList'!A1:D200,""); IFERROR(IF('_Import Pricey FtdList'!A1:A200="","","Pricey"),""), IFERROR('_Import Pricey FtdList'!A1:D200,""); IFERROR(IF('_Import Seanok FtdList'!A1:A200="","","Seanok"),""), IFERROR('_Import Seanok FtdList'!A1:D200,""); IFERROR(IF('_Import Gwen FtdList'!A1:A200="","","Gwen"),""), IFERROR('_Import Gwen FtdList'!A1:D200,""); IFERROR(IF('_Import Miko FtdList'!A1:A200="","","Miko"),""), IFERROR('_Import Miko FtdList'!A1:D200,""); IFERROR(IF('_Import Concept FtdList'!A1:A200="","","Concept"),""), IFERROR('_Import Concept FtdList'!A1:D200,""); IFERROR(IF('_Import Daily FtdList'!A1:A200="","","Daily"),""), IFERROR('_Import Daily FtdList'!A1:D200,""); IFERROR(IF('_Import Prime FtdList'!A1:A200="","","Prime"),""), IFERROR('_Import Prime FtdList'!A1:D200,""); IFERROR(IF('_Import Yuri FtdList'!A1:A200="","","Yuri"),""), IFERROR('_Import Yuri FtdList'!A1:D200,"")}, {IFERROR('_Import Tuna FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Plat FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Chella FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Moneyheist FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Seb FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Pricey FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Seanok FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Gwen FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Miko FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Concept FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Daily FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Prime FtdList'!A1:A200&lt;&gt;"",FALSE); IFERROR('_Import Yuri FtdList'!A1:A200&lt;&gt;"",FALSE)}), "")</f>
         <v/>
       </c>
       <c r="D5" s="8" t="n"/>
@@ -27414,7 +27414,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!B4:B203"),IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!AC4:AC203"),IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!W4:W203"),IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!B4:B203"),IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!AC4:AC203"),IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!W4:W203"),IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -27434,7 +27434,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Moneyheist - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -27454,7 +27454,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1zjxFDteeU3YWlO9w9B92o-2ol3_yJiNnttovezeMnOg", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -27474,7 +27474,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -27494,7 +27494,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -27514,7 +27514,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!B4:B203"),IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!AC4:AC203"),IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!W4:W203"),IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!B4:B203"),IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!AC4:AC203"),IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!W4:W203"),IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -27534,7 +27534,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Seb - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -27554,7 +27554,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZWfAr3sHXFGpNgieFKycyZq0GxTNMJTcAG668Pk15rg", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -27574,7 +27574,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -27594,7 +27594,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -27700,7 +27700,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <f>SORT(IFERROR(FILTER({IFERROR(IF('_Import Yuri Book'!B1:B200="","","Yuri"),""), IFERROR('_Import Yuri Book'!B1:F200,""), IFERROR(IFERROR('_Import Yuri VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Yuri VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Yuri VIPTeam'!C1:C200,""),IFERROR('_Import Yuri VIPTeam'!D1:D200,"")),""), IFERROR('_Import Yuri Book'!I1:K200,""); IFERROR(IF('_Import Tuna Book'!B1:B200="","","Tuna"),""), IFERROR('_Import Tuna Book'!B1:F200,""), IFERROR(IFERROR('_Import Tuna VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Tuna VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Tuna VIPTeam'!C1:C200,""),IFERROR('_Import Tuna VIPTeam'!D1:D200,"")),""), IFERROR('_Import Tuna Book'!I1:K200,""); IFERROR(IF('_Import Plat Book'!B1:B200="","","Plat"),""), IFERROR('_Import Plat Book'!B1:F200,""), IFERROR(IFERROR('_Import Plat VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Plat VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Plat VIPTeam'!C1:C200,""),IFERROR('_Import Plat VIPTeam'!D1:D200,"")),""), IFERROR('_Import Plat Book'!I1:K200,""); IFERROR(IF('_Import Chella Book'!B1:B200="","","Chella"),""), IFERROR('_Import Chella Book'!B1:F200,""), IFERROR(IFERROR('_Import Chella VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Chella VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Chella VIPTeam'!C1:C200,""),IFERROR('_Import Chella VIPTeam'!D1:D200,"")),""), IFERROR('_Import Chella Book'!I1:K200,""); IFERROR(IF('_Import Moneyheist Book'!B1:B200="","","Moneyheist"),""), IFERROR('_Import Moneyheist Book'!B1:F200,""), IFERROR(IFERROR('_Import Moneyheist VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Moneyheist VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Moneyheist VIPTeam'!C1:C200,""),IFERROR('_Import Moneyheist VIPTeam'!D1:D200,"")),""), IFERROR('_Import Moneyheist Book'!I1:K200,""); IFERROR(IF('_Import Seb Book'!B1:B200="","","Seb"),""), IFERROR('_Import Seb Book'!B1:F200,""), IFERROR(IFERROR('_Import Seb VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Seb VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Seb VIPTeam'!C1:C200,""),IFERROR('_Import Seb VIPTeam'!D1:D200,"")),""), IFERROR('_Import Seb Book'!I1:K200,""); IFERROR(IF('_Import Pricey Book'!B1:B200="","","Pricey"),""), IFERROR('_Import Pricey Book'!B1:F200,""), IFERROR(IFERROR('_Import Pricey VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Pricey VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Pricey VIPTeam'!C1:C200,""),IFERROR('_Import Pricey VIPTeam'!D1:D200,"")),""), IFERROR('_Import Pricey Book'!I1:K200,""); IFERROR(IF('_Import Seanok Book'!B1:B200="","","Seanok"),""), IFERROR('_Import Seanok Book'!B1:F200,""), IFERROR(IFERROR('_Import Seanok VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Seanok VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Seanok VIPTeam'!C1:C200,""),IFERROR('_Import Seanok VIPTeam'!D1:D200,"")),""), IFERROR('_Import Seanok Book'!I1:K200,""); IFERROR(IF('_Import Gwen Book'!B1:B200="","","Gwen"),""), IFERROR('_Import Gwen Book'!B1:F200,""), IFERROR(IFERROR('_Import Gwen VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Gwen VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Gwen VIPTeam'!C1:C200,""),IFERROR('_Import Gwen VIPTeam'!D1:D200,"")),""), IFERROR('_Import Gwen Book'!I1:K200,""); IFERROR(IF('_Import Miko Book'!B1:B200="","","Miko"),""), IFERROR('_Import Miko Book'!B1:F200,""), IFERROR(IFERROR('_Import Miko VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Miko VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Miko VIPTeam'!C1:C200,""),IFERROR('_Import Miko VIPTeam'!D1:D200,"")),""), IFERROR('_Import Miko Book'!I1:K200,""); IFERROR(IF('_Import Concept Book'!B1:B200="","","Concept"),""), IFERROR('_Import Concept Book'!B1:F200,""), IFERROR(IFERROR('_Import Concept VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Concept VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Concept VIPTeam'!C1:C200,""),IFERROR('_Import Concept VIPTeam'!D1:D200,"")),""), IFERROR('_Import Concept Book'!I1:K200,""); IFERROR(IF('_Import Daily Book'!B1:B200="","","Daily"),""), IFERROR('_Import Daily Book'!B1:F200,""), IFERROR(IFERROR('_Import Daily VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Daily VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Daily VIPTeam'!C1:C200,""),IFERROR('_Import Daily VIPTeam'!D1:D200,"")),""), IFERROR('_Import Daily Book'!I1:K200,""); IFERROR(IF('_Import Prime Book'!B1:B200="","","Prime"),""), IFERROR('_Import Prime Book'!B1:F200,""), IFERROR(IFERROR('_Import Prime VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Prime VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Prime VIPTeam'!C1:C200,""),IFERROR('_Import Prime VIPTeam'!D1:D200,"")),""), IFERROR('_Import Prime Book'!I1:K200,"")}, {IFERROR((('_Import Yuri Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Yuri VIPTeam'!B1:B200,"")="Yes"))*('_Import Yuri Book'!B1:B200&lt;&gt;"")*('_Import Yuri Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Tuna Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Tuna VIPTeam'!B1:B200,"")="Yes"))*('_Import Tuna Book'!B1:B200&lt;&gt;"")*('_Import Tuna Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Plat Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Plat VIPTeam'!B1:B200,"")="Yes"))*('_Import Plat Book'!B1:B200&lt;&gt;"")*('_Import Plat Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Chella Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Chella VIPTeam'!B1:B200,"")="Yes"))*('_Import Chella Book'!B1:B200&lt;&gt;"")*('_Import Chella Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Moneyheist Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Moneyheist VIPTeam'!B1:B200,"")="Yes"))*('_Import Moneyheist Book'!B1:B200&lt;&gt;"")*('_Import Moneyheist Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Seb Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Seb VIPTeam'!B1:B200,"")="Yes"))*('_Import Seb Book'!B1:B200&lt;&gt;"")*('_Import Seb Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Pricey Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Pricey VIPTeam'!B1:B200,"")="Yes"))*('_Import Pricey Book'!B1:B200&lt;&gt;"")*('_Import Pricey Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Seanok Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Seanok VIPTeam'!B1:B200,"")="Yes"))*('_Import Seanok Book'!B1:B200&lt;&gt;"")*('_Import Seanok Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Gwen Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Gwen VIPTeam'!B1:B200,"")="Yes"))*('_Import Gwen Book'!B1:B200&lt;&gt;"")*('_Import Gwen Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Miko Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Miko VIPTeam'!B1:B200,"")="Yes"))*('_Import Miko Book'!B1:B200&lt;&gt;"")*('_Import Miko Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Concept Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Concept VIPTeam'!B1:B200,"")="Yes"))*('_Import Concept Book'!B1:B200&lt;&gt;"")*('_Import Concept Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Daily Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Daily VIPTeam'!B1:B200,"")="Yes"))*('_Import Daily Book'!B1:B200&lt;&gt;"")*('_Import Daily Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Prime Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Prime VIPTeam'!B1:B200,"")="Yes"))*('_Import Prime Book'!B1:B200&lt;&gt;"")*('_Import Prime Book'!D1:D200&lt;&gt;""),FALSE)}), ""), 8, FALSE)</f>
+        <f>SORT(IFERROR(FILTER({IFERROR(IF('_Import Tuna Book'!B1:B200="","","Tuna"),""), IFERROR('_Import Tuna Book'!B1:F200,""), IFERROR(IFERROR('_Import Tuna VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Tuna VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Tuna VIPTeam'!C1:C200,""),IFERROR('_Import Tuna VIPTeam'!D1:D200,"")),""), IFERROR('_Import Tuna Book'!I1:K200,""); IFERROR(IF('_Import Plat Book'!B1:B200="","","Plat"),""), IFERROR('_Import Plat Book'!B1:F200,""), IFERROR(IFERROR('_Import Plat VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Plat VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Plat VIPTeam'!C1:C200,""),IFERROR('_Import Plat VIPTeam'!D1:D200,"")),""), IFERROR('_Import Plat Book'!I1:K200,""); IFERROR(IF('_Import Chella Book'!B1:B200="","","Chella"),""), IFERROR('_Import Chella Book'!B1:F200,""), IFERROR(IFERROR('_Import Chella VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Chella VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Chella VIPTeam'!C1:C200,""),IFERROR('_Import Chella VIPTeam'!D1:D200,"")),""), IFERROR('_Import Chella Book'!I1:K200,""); IFERROR(IF('_Import Moneyheist Book'!B1:B200="","","Moneyheist"),""), IFERROR('_Import Moneyheist Book'!B1:F200,""), IFERROR(IFERROR('_Import Moneyheist VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Moneyheist VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Moneyheist VIPTeam'!C1:C200,""),IFERROR('_Import Moneyheist VIPTeam'!D1:D200,"")),""), IFERROR('_Import Moneyheist Book'!I1:K200,""); IFERROR(IF('_Import Seb Book'!B1:B200="","","Seb"),""), IFERROR('_Import Seb Book'!B1:F200,""), IFERROR(IFERROR('_Import Seb VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Seb VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Seb VIPTeam'!C1:C200,""),IFERROR('_Import Seb VIPTeam'!D1:D200,"")),""), IFERROR('_Import Seb Book'!I1:K200,""); IFERROR(IF('_Import Pricey Book'!B1:B200="","","Pricey"),""), IFERROR('_Import Pricey Book'!B1:F200,""), IFERROR(IFERROR('_Import Pricey VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Pricey VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Pricey VIPTeam'!C1:C200,""),IFERROR('_Import Pricey VIPTeam'!D1:D200,"")),""), IFERROR('_Import Pricey Book'!I1:K200,""); IFERROR(IF('_Import Seanok Book'!B1:B200="","","Seanok"),""), IFERROR('_Import Seanok Book'!B1:F200,""), IFERROR(IFERROR('_Import Seanok VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Seanok VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Seanok VIPTeam'!C1:C200,""),IFERROR('_Import Seanok VIPTeam'!D1:D200,"")),""), IFERROR('_Import Seanok Book'!I1:K200,""); IFERROR(IF('_Import Gwen Book'!B1:B200="","","Gwen"),""), IFERROR('_Import Gwen Book'!B1:F200,""), IFERROR(IFERROR('_Import Gwen VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Gwen VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Gwen VIPTeam'!C1:C200,""),IFERROR('_Import Gwen VIPTeam'!D1:D200,"")),""), IFERROR('_Import Gwen Book'!I1:K200,""); IFERROR(IF('_Import Miko Book'!B1:B200="","","Miko"),""), IFERROR('_Import Miko Book'!B1:F200,""), IFERROR(IFERROR('_Import Miko VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Miko VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Miko VIPTeam'!C1:C200,""),IFERROR('_Import Miko VIPTeam'!D1:D200,"")),""), IFERROR('_Import Miko Book'!I1:K200,""); IFERROR(IF('_Import Concept Book'!B1:B200="","","Concept"),""), IFERROR('_Import Concept Book'!B1:F200,""), IFERROR(IFERROR('_Import Concept VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Concept VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Concept VIPTeam'!C1:C200,""),IFERROR('_Import Concept VIPTeam'!D1:D200,"")),""), IFERROR('_Import Concept Book'!I1:K200,""); IFERROR(IF('_Import Daily Book'!B1:B200="","","Daily"),""), IFERROR('_Import Daily Book'!B1:F200,""), IFERROR(IFERROR('_Import Daily VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Daily VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Daily VIPTeam'!C1:C200,""),IFERROR('_Import Daily VIPTeam'!D1:D200,"")),""), IFERROR('_Import Daily Book'!I1:K200,""); IFERROR(IF('_Import Prime Book'!B1:B200="","","Prime"),""), IFERROR('_Import Prime Book'!B1:F200,""), IFERROR(IFERROR('_Import Prime VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Prime VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Prime VIPTeam'!C1:C200,""),IFERROR('_Import Prime VIPTeam'!D1:D200,"")),""), IFERROR('_Import Prime Book'!I1:K200,""); IFERROR(IF('_Import Yuri Book'!B1:B200="","","Yuri"),""), IFERROR('_Import Yuri Book'!B1:F200,""), IFERROR(IFERROR('_Import Yuri VIPTeam'!B1:B200,""),""), IFERROR(IF(IFERROR('_Import Yuri VIPTeam'!C1:C200,"")&lt;&gt;"",IFERROR('_Import Yuri VIPTeam'!C1:C200,""),IFERROR('_Import Yuri VIPTeam'!D1:D200,"")),""), IFERROR('_Import Yuri Book'!I1:K200,"")}, {IFERROR((('_Import Tuna Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Tuna VIPTeam'!B1:B200,"")="Yes"))*('_Import Tuna Book'!B1:B200&lt;&gt;"")*('_Import Tuna Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Plat Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Plat VIPTeam'!B1:B200,"")="Yes"))*('_Import Plat Book'!B1:B200&lt;&gt;"")*('_Import Plat Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Chella Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Chella VIPTeam'!B1:B200,"")="Yes"))*('_Import Chella Book'!B1:B200&lt;&gt;"")*('_Import Chella Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Moneyheist Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Moneyheist VIPTeam'!B1:B200,"")="Yes"))*('_Import Moneyheist Book'!B1:B200&lt;&gt;"")*('_Import Moneyheist Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Seb Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Seb VIPTeam'!B1:B200,"")="Yes"))*('_Import Seb Book'!B1:B200&lt;&gt;"")*('_Import Seb Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Pricey Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Pricey VIPTeam'!B1:B200,"")="Yes"))*('_Import Pricey Book'!B1:B200&lt;&gt;"")*('_Import Pricey Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Seanok Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Seanok VIPTeam'!B1:B200,"")="Yes"))*('_Import Seanok Book'!B1:B200&lt;&gt;"")*('_Import Seanok Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Gwen Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Gwen VIPTeam'!B1:B200,"")="Yes"))*('_Import Gwen Book'!B1:B200&lt;&gt;"")*('_Import Gwen Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Miko Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Miko VIPTeam'!B1:B200,"")="Yes"))*('_Import Miko Book'!B1:B200&lt;&gt;"")*('_Import Miko Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Concept Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Concept VIPTeam'!B1:B200,"")="Yes"))*('_Import Concept Book'!B1:B200&lt;&gt;"")*('_Import Concept Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Daily Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Daily VIPTeam'!B1:B200,"")="Yes"))*('_Import Daily Book'!B1:B200&lt;&gt;"")*('_Import Daily Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Prime Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Prime VIPTeam'!B1:B200,"")="Yes"))*('_Import Prime Book'!B1:B200&lt;&gt;"")*('_Import Prime Book'!D1:D200&lt;&gt;""),FALSE); IFERROR((('_Import Yuri Book'!E1:E200="VIP Transferred")+(IFERROR('_Import Yuri VIPTeam'!B1:B200,"")="Yes"))*('_Import Yuri Book'!B1:B200&lt;&gt;"")*('_Import Yuri Book'!D1:D200&lt;&gt;""),FALSE)}), ""), 8, FALSE)</f>
         <v/>
       </c>
       <c r="H5" s="8" t="n"/>
@@ -40724,7 +40724,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!B4:B203"),IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!AC4:AC203"),IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!W4:W203"),IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!B4:B203"),IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!AC4:AC203"),IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!W4:W203"),IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -40744,7 +40744,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Pricey - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -40764,7 +40764,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1ZU7EXQAHws9qptiNUTqPi6fKE1ALTdipfU-gSaNNUAk", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -40784,7 +40784,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -40804,7 +40804,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -40824,7 +40824,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!B4:B203"),IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!AC4:AC203"),IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!W4:W203"),IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!B4:B203"),IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!AC4:AC203"),IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!W4:W203"),IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -40844,7 +40844,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Seanok - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -40864,7 +40864,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1e0krwNw2H4hns9MSex-7cGvwH7epyhkKIxvVfT9Svu4", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -40884,7 +40884,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -40904,7 +40904,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -40984,7 +40984,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <f>IFERROR(FILTER({IF('_Import Yuri Book'!B1:B200="","","Yuri"), '_Import Yuri Book'!B1:B200, '_Import Yuri Book'!E1:F200, '_Import Yuri Book'!I1:K200; IF('_Import Tuna Book'!B1:B200="","","Tuna"), '_Import Tuna Book'!B1:B200, '_Import Tuna Book'!E1:F200, '_Import Tuna Book'!I1:K200; IF('_Import Plat Book'!B1:B200="","","Plat"), '_Import Plat Book'!B1:B200, '_Import Plat Book'!E1:F200, '_Import Plat Book'!I1:K200; IF('_Import Chella Book'!B1:B200="","","Chella"), '_Import Chella Book'!B1:B200, '_Import Chella Book'!E1:F200, '_Import Chella Book'!I1:K200; IF('_Import Moneyheist Book'!B1:B200="","","Moneyheist"), '_Import Moneyheist Book'!B1:B200, '_Import Moneyheist Book'!E1:F200, '_Import Moneyheist Book'!I1:K200; IF('_Import Seb Book'!B1:B200="","","Seb"), '_Import Seb Book'!B1:B200, '_Import Seb Book'!E1:F200, '_Import Seb Book'!I1:K200; IF('_Import Pricey Book'!B1:B200="","","Pricey"), '_Import Pricey Book'!B1:B200, '_Import Pricey Book'!E1:F200, '_Import Pricey Book'!I1:K200; IF('_Import Seanok Book'!B1:B200="","","Seanok"), '_Import Seanok Book'!B1:B200, '_Import Seanok Book'!E1:F200, '_Import Seanok Book'!I1:K200; IF('_Import Gwen Book'!B1:B200="","","Gwen"), '_Import Gwen Book'!B1:B200, '_Import Gwen Book'!E1:F200, '_Import Gwen Book'!I1:K200; IF('_Import Miko Book'!B1:B200="","","Miko"), '_Import Miko Book'!B1:B200, '_Import Miko Book'!E1:F200, '_Import Miko Book'!I1:K200; IF('_Import Concept Book'!B1:B200="","","Concept"), '_Import Concept Book'!B1:B200, '_Import Concept Book'!E1:F200, '_Import Concept Book'!I1:K200; IF('_Import Daily Book'!B1:B200="","","Daily"), '_Import Daily Book'!B1:B200, '_Import Daily Book'!E1:F200, '_Import Daily Book'!I1:K200; IF('_Import Prime Book'!B1:B200="","","Prime"), '_Import Prime Book'!B1:B200, '_Import Prime Book'!E1:F200, '_Import Prime Book'!I1:K200}, {(('_Import Yuri Book'!J1:J200&lt;&gt;"")*('_Import Yuri Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Tuna Book'!J1:J200&lt;&gt;"")*('_Import Tuna Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Plat Book'!J1:J200&lt;&gt;"")*('_Import Plat Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Chella Book'!J1:J200&lt;&gt;"")*('_Import Chella Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Moneyheist Book'!J1:J200&lt;&gt;"")*('_Import Moneyheist Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Seb Book'!J1:J200&lt;&gt;"")*('_Import Seb Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Pricey Book'!J1:J200&lt;&gt;"")*('_Import Pricey Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Seanok Book'!J1:J200&lt;&gt;"")*('_Import Seanok Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Gwen Book'!J1:J200&lt;&gt;"")*('_Import Gwen Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Miko Book'!J1:J200&lt;&gt;"")*('_Import Miko Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Concept Book'!J1:J200&lt;&gt;"")*('_Import Concept Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Daily Book'!J1:J200&lt;&gt;"")*('_Import Daily Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Prime Book'!J1:J200&lt;&gt;"")*('_Import Prime Book'!J1:J200&lt;TODAY()))&gt;0}), "")</f>
+        <f>IFERROR(FILTER({IF('_Import Tuna Book'!B1:B200="","","Tuna"), '_Import Tuna Book'!B1:B200, '_Import Tuna Book'!E1:F200, '_Import Tuna Book'!I1:K200; IF('_Import Plat Book'!B1:B200="","","Plat"), '_Import Plat Book'!B1:B200, '_Import Plat Book'!E1:F200, '_Import Plat Book'!I1:K200; IF('_Import Chella Book'!B1:B200="","","Chella"), '_Import Chella Book'!B1:B200, '_Import Chella Book'!E1:F200, '_Import Chella Book'!I1:K200; IF('_Import Moneyheist Book'!B1:B200="","","Moneyheist"), '_Import Moneyheist Book'!B1:B200, '_Import Moneyheist Book'!E1:F200, '_Import Moneyheist Book'!I1:K200; IF('_Import Seb Book'!B1:B200="","","Seb"), '_Import Seb Book'!B1:B200, '_Import Seb Book'!E1:F200, '_Import Seb Book'!I1:K200; IF('_Import Pricey Book'!B1:B200="","","Pricey"), '_Import Pricey Book'!B1:B200, '_Import Pricey Book'!E1:F200, '_Import Pricey Book'!I1:K200; IF('_Import Seanok Book'!B1:B200="","","Seanok"), '_Import Seanok Book'!B1:B200, '_Import Seanok Book'!E1:F200, '_Import Seanok Book'!I1:K200; IF('_Import Gwen Book'!B1:B200="","","Gwen"), '_Import Gwen Book'!B1:B200, '_Import Gwen Book'!E1:F200, '_Import Gwen Book'!I1:K200; IF('_Import Miko Book'!B1:B200="","","Miko"), '_Import Miko Book'!B1:B200, '_Import Miko Book'!E1:F200, '_Import Miko Book'!I1:K200; IF('_Import Concept Book'!B1:B200="","","Concept"), '_Import Concept Book'!B1:B200, '_Import Concept Book'!E1:F200, '_Import Concept Book'!I1:K200; IF('_Import Daily Book'!B1:B200="","","Daily"), '_Import Daily Book'!B1:B200, '_Import Daily Book'!E1:F200, '_Import Daily Book'!I1:K200; IF('_Import Prime Book'!B1:B200="","","Prime"), '_Import Prime Book'!B1:B200, '_Import Prime Book'!E1:F200, '_Import Prime Book'!I1:K200; IF('_Import Yuri Book'!B1:B200="","","Yuri"), '_Import Yuri Book'!B1:B200, '_Import Yuri Book'!E1:F200, '_Import Yuri Book'!I1:K200}, {(('_Import Tuna Book'!J1:J200&lt;&gt;"")*('_Import Tuna Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Plat Book'!J1:J200&lt;&gt;"")*('_Import Plat Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Chella Book'!J1:J200&lt;&gt;"")*('_Import Chella Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Moneyheist Book'!J1:J200&lt;&gt;"")*('_Import Moneyheist Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Seb Book'!J1:J200&lt;&gt;"")*('_Import Seb Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Pricey Book'!J1:J200&lt;&gt;"")*('_Import Pricey Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Seanok Book'!J1:J200&lt;&gt;"")*('_Import Seanok Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Gwen Book'!J1:J200&lt;&gt;"")*('_Import Gwen Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Miko Book'!J1:J200&lt;&gt;"")*('_Import Miko Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Concept Book'!J1:J200&lt;&gt;"")*('_Import Concept Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Daily Book'!J1:J200&lt;&gt;"")*('_Import Daily Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Prime Book'!J1:J200&lt;&gt;"")*('_Import Prime Book'!J1:J200&lt;TODAY()))&gt;0; (('_Import Yuri Book'!J1:J200&lt;&gt;"")*('_Import Yuri Book'!J1:J200&lt;TODAY()))&gt;0}), "")</f>
         <v/>
       </c>
       <c r="E5" s="8" t="n"/>
@@ -51408,7 +51408,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!B4:B203"),IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!AC4:AC203"),IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!W4:W203"),IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!B4:B203"),IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!AC4:AC203"),IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!W4:W203"),IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -51428,7 +51428,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Gwen - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -51448,7 +51448,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1PusLuNTxs7n2kCQJRCD1K0XnSwrpBZDaelz51bcEho0", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -51468,7 +51468,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -51488,7 +51488,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -51508,7 +51508,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!B4:B203"),IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!AC4:AC203"),IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!W4:W203"),IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!B4:B203"),IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!AC4:AC203"),IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!W4:W203"),IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -51528,7 +51528,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Miko - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -51548,7 +51548,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1GElB1aCPsITtPtn-ebNIPW9fxj5czH-H8Tzvo0umY4Y", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -51568,7 +51568,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -51588,7 +51588,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -51679,7 +51679,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTIF('_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Plat ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Chella ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Moneyheist ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Seb ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Pricey ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Seanok ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Gwen ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Miko ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Concept ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Daily ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Prime ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <f>COUNTIF('_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Plat ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Chella ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Moneyheist ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Seb ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Pricey ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Seanok ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Gwen ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Miko ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Concept ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Daily ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Prime ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")+COUNTIF('_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIF('_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -51688,7 +51688,7 @@
         </is>
       </c>
       <c r="E7" s="14">
-        <f>COUNTIF('_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <f>COUNTIF('_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")+COUNTIF('_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
@@ -51739,403 +51739,403 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Yuri</t>
+          <t>Tuna</t>
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS('_Import Yuri Book'!$H$1:$H$200,TODAY(),'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
+        <f>COUNTIFS('_Import Tuna Book'!$H$1:$H$200,TODAY(),'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Yuri",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
+        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Tuna",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Yuri",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
+        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Tuna",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
       <c r="F11" s="16">
-        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
       <c r="G11" s="16">
-        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Yuri",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Tuna</t>
-        </is>
-      </c>
-      <c r="B12" s="16">
-        <f>COUNTIFS('_Import Tuna Book'!$H$1:$H$200,TODAY(),'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
-        <v/>
-      </c>
-      <c r="C12" s="16">
-        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Tuna",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
-        <v/>
-      </c>
-      <c r="D12" s="16">
-        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
-        <v/>
-      </c>
-      <c r="E12" s="16">
-        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Tuna",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
-        <v/>
-      </c>
-      <c r="F12" s="16">
-        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
-        <v/>
-      </c>
-      <c r="G12" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Tuna",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Plat</t>
         </is>
       </c>
-      <c r="B13" s="16">
+      <c r="B12" s="16">
         <f>COUNTIFS('_Import Plat Book'!$H$1:$H$200,TODAY(),'_Import Plat Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Plat Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C13" s="16">
+      <c r="C12" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Plat",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D13" s="16">
+      <c r="D12" s="16">
         <f>COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E12" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Plat",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F12" s="16">
         <f>COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G13" s="16">
+      <c r="G12" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Plat",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Chella</t>
         </is>
       </c>
-      <c r="B14" s="16">
+      <c r="B13" s="16">
         <f>COUNTIFS('_Import Chella Book'!$H$1:$H$200,TODAY(),'_Import Chella Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Chella Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C14" s="16">
+      <c r="C13" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Chella",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D14" s="16">
+      <c r="D13" s="16">
         <f>COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E14" s="16">
+      <c r="E13" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Chella",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F14" s="16">
+      <c r="F13" s="16">
         <f>COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G14" s="16">
+      <c r="G13" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Chella",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Moneyheist</t>
         </is>
       </c>
-      <c r="B15" s="16">
+      <c r="B14" s="16">
         <f>COUNTIFS('_Import Moneyheist Book'!$H$1:$H$200,TODAY(),'_Import Moneyheist Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Moneyheist Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C15" s="16">
+      <c r="C14" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Moneyheist",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D15" s="16">
+      <c r="D14" s="16">
         <f>COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E14" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Moneyheist",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F14" s="16">
         <f>COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G15" s="16">
+      <c r="G14" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Moneyheist",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Seb</t>
         </is>
       </c>
-      <c r="B16" s="16">
+      <c r="B15" s="16">
         <f>COUNTIFS('_Import Seb Book'!$H$1:$H$200,TODAY(),'_Import Seb Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Seb Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C16" s="16">
+      <c r="C15" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Seb",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D16" s="16">
+      <c r="D15" s="16">
         <f>COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E15" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Seb",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F16" s="16">
+      <c r="F15" s="16">
         <f>COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G16" s="16">
+      <c r="G15" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Seb",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Pricey</t>
         </is>
       </c>
-      <c r="B17" s="16">
+      <c r="B16" s="16">
         <f>COUNTIFS('_Import Pricey Book'!$H$1:$H$200,TODAY(),'_Import Pricey Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Pricey Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C17" s="16">
+      <c r="C16" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Pricey",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D17" s="16">
+      <c r="D16" s="16">
         <f>COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E17" s="16">
+      <c r="E16" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Pricey",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F17" s="16">
+      <c r="F16" s="16">
         <f>COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G17" s="16">
+      <c r="G16" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Pricey",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Seanok</t>
         </is>
       </c>
-      <c r="B18" s="16">
+      <c r="B17" s="16">
         <f>COUNTIFS('_Import Seanok Book'!$H$1:$H$200,TODAY(),'_Import Seanok Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Seanok Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C18" s="16">
+      <c r="C17" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Seanok",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D18" s="16">
+      <c r="D17" s="16">
         <f>COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E18" s="16">
+      <c r="E17" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Seanok",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F18" s="16">
+      <c r="F17" s="16">
         <f>COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G18" s="16">
+      <c r="G17" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Seanok",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Gwen</t>
         </is>
       </c>
-      <c r="B19" s="16">
+      <c r="B18" s="16">
         <f>COUNTIFS('_Import Gwen Book'!$H$1:$H$200,TODAY(),'_Import Gwen Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Gwen Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C19" s="16">
+      <c r="C18" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Gwen",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D19" s="16">
+      <c r="D18" s="16">
         <f>COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E19" s="16">
+      <c r="E18" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Gwen",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F19" s="16">
+      <c r="F18" s="16">
         <f>COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G19" s="16">
+      <c r="G18" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Gwen",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Miko</t>
         </is>
       </c>
-      <c r="B20" s="16">
+      <c r="B19" s="16">
         <f>COUNTIFS('_Import Miko Book'!$H$1:$H$200,TODAY(),'_Import Miko Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Miko Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C20" s="16">
+      <c r="C19" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Miko",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D20" s="16">
+      <c r="D19" s="16">
         <f>COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E20" s="16">
+      <c r="E19" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Miko",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F20" s="16">
+      <c r="F19" s="16">
         <f>COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G20" s="16">
+      <c r="G19" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Miko",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Concept</t>
         </is>
       </c>
-      <c r="B21" s="16">
+      <c r="B20" s="16">
         <f>COUNTIFS('_Import Concept Book'!$H$1:$H$200,TODAY(),'_Import Concept Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Concept Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C21" s="16">
+      <c r="C20" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Concept",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D21" s="16">
+      <c r="D20" s="16">
         <f>COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E21" s="16">
+      <c r="E20" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Concept",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F21" s="16">
+      <c r="F20" s="16">
         <f>COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G21" s="16">
+      <c r="G20" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Concept",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="B22" s="16">
+      <c r="B21" s="16">
         <f>COUNTIFS('_Import Daily Book'!$H$1:$H$200,TODAY(),'_Import Daily Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Daily Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C22" s="16">
+      <c r="C21" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Daily",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D22" s="16">
+      <c r="D21" s="16">
         <f>COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E22" s="16">
+      <c r="E21" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Daily",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F22" s="16">
+      <c r="F21" s="16">
         <f>COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="G22" s="16">
+      <c r="G21" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Daily",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Prime</t>
         </is>
       </c>
-      <c r="B23" s="16">
+      <c r="B22" s="16">
         <f>COUNTIFS('_Import Prime Book'!$H$1:$H$200,TODAY(),'_Import Prime Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Prime Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C23" s="16">
+      <c r="C22" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Prime",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="D23" s="16">
+      <c r="D22" s="16">
         <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="E23" s="16">
+      <c r="E22" s="16">
         <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Prime",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
-      <c r="F23" s="16">
+      <c r="F22" s="16">
         <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
+      <c r="G22" s="16">
+        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Prime",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Yuri</t>
+        </is>
+      </c>
+      <c r="B23" s="16">
+        <f>COUNTIFS('_Import Yuri Book'!$H$1:$H$200,TODAY(),'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
+        <v/>
+      </c>
+      <c r="C23" s="16">
+        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$E$5:$E$17,MATCH("Yuri",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
+        <v/>
+      </c>
+      <c r="D23" s="16">
+        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <v/>
+      </c>
+      <c r="E23" s="16">
+        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$F$5:$F$17,MATCH("Yuri",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
+        <v/>
+      </c>
+      <c r="F23" s="16">
+        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <v/>
+      </c>
       <c r="G23" s="16">
-        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Prime",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
+        <f>IFERROR(INDEX('Team &amp; KPI Targets'!$G$5:$G$17,MATCH("Yuri",'Team &amp; KPI Targets'!$A$5:$A$17,0)),"TBD")</f>
         <v/>
       </c>
     </row>
@@ -52217,403 +52217,403 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Yuri</t>
+          <t>Tuna</t>
         </is>
       </c>
       <c r="B28" s="16">
-        <f>COUNTIFS('_Import Yuri Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
+        <f>COUNTIFS('_Import Tuna Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
       <c r="C28" s="16">
-        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
       <c r="D28" s="16">
-        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
       <c r="E28" s="16">
-        <f>COUNTIFS('_Import Yuri Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
+        <f>COUNTIFS('_Import Tuna Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
       <c r="F28" s="16">
-        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
       <c r="G28" s="16">
-        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>Tuna</t>
-        </is>
-      </c>
-      <c r="B29" s="16">
-        <f>COUNTIFS('_Import Tuna Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
-        <v/>
-      </c>
-      <c r="C29" s="16">
-        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
-        <v/>
-      </c>
-      <c r="D29" s="16">
-        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
-        <v/>
-      </c>
-      <c r="E29" s="16">
-        <f>COUNTIFS('_Import Tuna Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Tuna Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
-        <v/>
-      </c>
-      <c r="F29" s="16">
-        <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
         <f>COUNTIFS('_Import Tuna ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Tuna ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Tuna ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Plat</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B29" s="16">
         <f>COUNTIFS('_Import Plat Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Plat Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Plat Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Plat Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C29" s="16">
         <f>COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Plat ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Plat ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D30" s="16">
+      <c r="D29" s="16">
         <f>COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Plat ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E30" s="16">
+      <c r="E29" s="16">
         <f>COUNTIFS('_Import Plat Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Plat Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Plat Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Plat Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F30" s="16">
+      <c r="F29" s="16">
         <f>COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Plat ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Plat ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G30" s="16">
+      <c r="G29" s="16">
         <f>COUNTIFS('_Import Plat ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Plat ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Plat ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="15" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Chella</t>
         </is>
       </c>
-      <c r="B31" s="16">
+      <c r="B30" s="16">
         <f>COUNTIFS('_Import Chella Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Chella Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Chella Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Chella Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C31" s="16">
+      <c r="C30" s="16">
         <f>COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Chella ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Chella ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D31" s="16">
+      <c r="D30" s="16">
         <f>COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Chella ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E31" s="16">
+      <c r="E30" s="16">
         <f>COUNTIFS('_Import Chella Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Chella Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Chella Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Chella Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F31" s="16">
+      <c r="F30" s="16">
         <f>COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Chella ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Chella ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G31" s="16">
+      <c r="G30" s="16">
         <f>COUNTIFS('_Import Chella ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Chella ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Chella ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Moneyheist</t>
         </is>
       </c>
-      <c r="B32" s="16">
+      <c r="B31" s="16">
         <f>COUNTIFS('_Import Moneyheist Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Moneyheist Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Moneyheist Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Moneyheist Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C32" s="16">
+      <c r="C31" s="16">
         <f>COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D32" s="16">
+      <c r="D31" s="16">
         <f>COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E32" s="16">
+      <c r="E31" s="16">
         <f>COUNTIFS('_Import Moneyheist Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Moneyheist Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Moneyheist Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Moneyheist Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F32" s="16">
+      <c r="F31" s="16">
         <f>COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G32" s="16">
+      <c r="G31" s="16">
         <f>COUNTIFS('_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Moneyheist ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Moneyheist ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Seb</t>
         </is>
       </c>
-      <c r="B33" s="16">
+      <c r="B32" s="16">
         <f>COUNTIFS('_Import Seb Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seb Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Seb Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Seb Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C33" s="16">
+      <c r="C32" s="16">
         <f>COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seb ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seb ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D33" s="16">
+      <c r="D32" s="16">
         <f>COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seb ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E33" s="16">
+      <c r="E32" s="16">
         <f>COUNTIFS('_Import Seb Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seb Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Seb Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Seb Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F33" s="16">
+      <c r="F32" s="16">
         <f>COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seb ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seb ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G33" s="16">
+      <c r="G32" s="16">
         <f>COUNTIFS('_Import Seb ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seb ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seb ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>Pricey</t>
         </is>
       </c>
-      <c r="B34" s="16">
+      <c r="B33" s="16">
         <f>COUNTIFS('_Import Pricey Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Pricey Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Pricey Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Pricey Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C34" s="16">
+      <c r="C33" s="16">
         <f>COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Pricey ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Pricey ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D34" s="16">
+      <c r="D33" s="16">
         <f>COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Pricey ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E34" s="16">
+      <c r="E33" s="16">
         <f>COUNTIFS('_Import Pricey Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Pricey Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Pricey Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Pricey Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F34" s="16">
+      <c r="F33" s="16">
         <f>COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Pricey ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Pricey ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G34" s="16">
+      <c r="G33" s="16">
         <f>COUNTIFS('_Import Pricey ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Pricey ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Pricey ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Seanok</t>
         </is>
       </c>
-      <c r="B35" s="16">
+      <c r="B34" s="16">
         <f>COUNTIFS('_Import Seanok Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seanok Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Seanok Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Seanok Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C35" s="16">
+      <c r="C34" s="16">
         <f>COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seanok ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seanok ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D35" s="16">
+      <c r="D34" s="16">
         <f>COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Seanok ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E35" s="16">
+      <c r="E34" s="16">
         <f>COUNTIFS('_Import Seanok Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seanok Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Seanok Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Seanok Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F35" s="16">
+      <c r="F34" s="16">
         <f>COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seanok ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seanok ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G35" s="16">
+      <c r="G34" s="16">
         <f>COUNTIFS('_Import Seanok ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Seanok ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Seanok ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Gwen</t>
         </is>
       </c>
-      <c r="B36" s="16">
+      <c r="B35" s="16">
         <f>COUNTIFS('_Import Gwen Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Gwen Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Gwen Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Gwen Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C36" s="16">
+      <c r="C35" s="16">
         <f>COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Gwen ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Gwen ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D36" s="16">
+      <c r="D35" s="16">
         <f>COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Gwen ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E36" s="16">
+      <c r="E35" s="16">
         <f>COUNTIFS('_Import Gwen Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Gwen Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Gwen Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Gwen Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F36" s="16">
+      <c r="F35" s="16">
         <f>COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Gwen ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Gwen ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G36" s="16">
+      <c r="G35" s="16">
         <f>COUNTIFS('_Import Gwen ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Gwen ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Gwen ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Miko</t>
         </is>
       </c>
-      <c r="B37" s="16">
+      <c r="B36" s="16">
         <f>COUNTIFS('_Import Miko Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Miko Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Miko Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Miko Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C37" s="16">
+      <c r="C36" s="16">
         <f>COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Miko ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Miko ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D37" s="16">
+      <c r="D36" s="16">
         <f>COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Miko ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E37" s="16">
+      <c r="E36" s="16">
         <f>COUNTIFS('_Import Miko Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Miko Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Miko Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Miko Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F37" s="16">
+      <c r="F36" s="16">
         <f>COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Miko ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Miko ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G37" s="16">
+      <c r="G36" s="16">
         <f>COUNTIFS('_Import Miko ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Miko ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Miko ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Concept</t>
         </is>
       </c>
-      <c r="B38" s="16">
+      <c r="B37" s="16">
         <f>COUNTIFS('_Import Concept Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Concept Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Concept Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Concept Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C38" s="16">
+      <c r="C37" s="16">
         <f>COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Concept ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Concept ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D38" s="16">
+      <c r="D37" s="16">
         <f>COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Concept ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E38" s="16">
+      <c r="E37" s="16">
         <f>COUNTIFS('_Import Concept Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Concept Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Concept Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Concept Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F38" s="16">
+      <c r="F37" s="16">
         <f>COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Concept ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Concept ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G38" s="16">
+      <c r="G37" s="16">
         <f>COUNTIFS('_Import Concept ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Concept ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Concept ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="B39" s="16">
+      <c r="B38" s="16">
         <f>COUNTIFS('_Import Daily Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Daily Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Daily Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Daily Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C39" s="16">
+      <c r="C38" s="16">
         <f>COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Daily ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Daily ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D39" s="16">
+      <c r="D38" s="16">
         <f>COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Daily ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E39" s="16">
+      <c r="E38" s="16">
         <f>COUNTIFS('_Import Daily Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Daily Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Daily Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Daily Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F39" s="16">
+      <c r="F38" s="16">
         <f>COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Daily ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Daily ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="G39" s="16">
+      <c r="G38" s="16">
         <f>COUNTIFS('_Import Daily ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Daily ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Daily ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="15" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Prime</t>
         </is>
       </c>
-      <c r="B40" s="16">
+      <c r="B39" s="16">
         <f>COUNTIFS('_Import Prime Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Prime Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Prime Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Prime Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="C40" s="16">
+      <c r="C39" s="16">
         <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
-      <c r="D40" s="16">
+      <c r="D39" s="16">
         <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
-      <c r="E40" s="16">
+      <c r="E39" s="16">
         <f>COUNTIFS('_Import Prime Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Prime Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Prime Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Prime Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
         <v/>
       </c>
-      <c r="F40" s="16">
+      <c r="F39" s="16">
         <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
         <v/>
       </c>
+      <c r="G39" s="16">
+        <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>Yuri</t>
+        </is>
+      </c>
+      <c r="B40" s="16">
+        <f>COUNTIFS('_Import Yuri Book'!$H$1:$H$200,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
+        <v/>
+      </c>
+      <c r="C40" s="16">
+        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <v/>
+      </c>
+      <c r="D40" s="16">
+        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <v/>
+      </c>
+      <c r="E40" s="16">
+        <f>COUNTIFS('_Import Yuri Book'!$H$1:$H$200,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri Book'!$H$1:$H$200,"&lt;="&amp;TODAY(),'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Dead Lead",'_Import Yuri Book'!$E$1:$E$200,"&lt;&gt;Potential Lead")</f>
+        <v/>
+      </c>
+      <c r="F40" s="16">
+        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"VIP Transfer")+COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; VIP Transferred")</f>
+        <v/>
+      </c>
       <c r="G40" s="16">
-        <f>COUNTIFS('_Import Prime ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Prime ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Prime ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
+        <f>COUNTIFS('_Import Yuri ActivityLog'!$A$1:$A$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'_Import Yuri ActivityLog'!$A$1:$A$5000,"&lt;="&amp;TODAY(),'_Import Yuri ActivityLog'!$C$1:$C$5000,"*-&gt; First Deposit")</f>
         <v/>
       </c>
     </row>
@@ -52657,7 +52657,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!B4:B203"),IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!AC4:AC203"),IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!W4:W203"),IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!B4:B203"),IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!AC4:AC203"),IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!W4:W203"),IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -52677,7 +52677,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Concept - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -52697,7 +52697,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("16XZ2V3L5SSrcuhjDDyxKYH5XX8HStG4sUWngBnRmDLo", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -52717,7 +52717,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -52737,7 +52737,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -52757,7 +52757,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!B4:B203"),IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!AC4:AC203"),IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!W4:W203"),IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!B4:B203"),IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!AC4:AC203"),IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!W4:W203"),IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -52777,7 +52777,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Daily - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -52797,7 +52797,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_5BmTcpK3SWziQWPleIrTcnfciVnNJS9prFkIbbHZzw", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -52817,7 +52817,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -52837,7 +52837,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>
@@ -52921,391 +52921,391 @@
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="19">
+        <f>IFERROR('_Import Tuna KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="19">
+        <f>IFERROR('_Import Tuna KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C5" s="19">
+        <f>IFERROR('_Import Tuna KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20">
+        <f>IFERROR('_Import Tuna KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E5" s="20">
+        <f>IFERROR('_Import Tuna KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="20">
+        <f>IFERROR('_Import Tuna KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="20">
+        <f>IFERROR('_Import Tuna KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="19">
+        <f>IFERROR('_Import Plat KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="19">
+        <f>IFERROR('_Import Plat KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C6" s="19">
+        <f>IFERROR('_Import Plat KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D6" s="20">
+        <f>IFERROR('_Import Plat KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E6" s="20">
+        <f>IFERROR('_Import Plat KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="20">
+        <f>IFERROR('_Import Plat KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="20">
+        <f>IFERROR('_Import Plat KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="19">
+        <f>IFERROR('_Import Chella KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B7" s="19">
+        <f>IFERROR('_Import Chella KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C7" s="19">
+        <f>IFERROR('_Import Chella KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D7" s="20">
+        <f>IFERROR('_Import Chella KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E7" s="20">
+        <f>IFERROR('_Import Chella KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="20">
+        <f>IFERROR('_Import Chella KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="20">
+        <f>IFERROR('_Import Chella KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="19">
+        <f>IFERROR('_Import Moneyheist KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B8" s="19">
+        <f>IFERROR('_Import Moneyheist KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>IFERROR('_Import Moneyheist KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="20">
+        <f>IFERROR('_Import Moneyheist KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="20">
+        <f>IFERROR('_Import Moneyheist KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="20">
+        <f>IFERROR('_Import Moneyheist KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="20">
+        <f>IFERROR('_Import Moneyheist KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="19">
+        <f>IFERROR('_Import Seb KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B9" s="19">
+        <f>IFERROR('_Import Seb KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C9" s="19">
+        <f>IFERROR('_Import Seb KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D9" s="20">
+        <f>IFERROR('_Import Seb KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E9" s="20">
+        <f>IFERROR('_Import Seb KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="20">
+        <f>IFERROR('_Import Seb KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="20">
+        <f>IFERROR('_Import Seb KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="19">
+        <f>IFERROR('_Import Pricey KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B10" s="19">
+        <f>IFERROR('_Import Pricey KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C10" s="19">
+        <f>IFERROR('_Import Pricey KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="20">
+        <f>IFERROR('_Import Pricey KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="20">
+        <f>IFERROR('_Import Pricey KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="20">
+        <f>IFERROR('_Import Pricey KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="20">
+        <f>IFERROR('_Import Pricey KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="19">
+        <f>IFERROR('_Import Seanok KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B11" s="19">
+        <f>IFERROR('_Import Seanok KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="19">
+        <f>IFERROR('_Import Seanok KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="20">
+        <f>IFERROR('_Import Seanok KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="20">
+        <f>IFERROR('_Import Seanok KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="20">
+        <f>IFERROR('_Import Seanok KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="20">
+        <f>IFERROR('_Import Seanok KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="19">
+        <f>IFERROR('_Import Gwen KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B12" s="19">
+        <f>IFERROR('_Import Gwen KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="19">
+        <f>IFERROR('_Import Gwen KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="20">
+        <f>IFERROR('_Import Gwen KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="20">
+        <f>IFERROR('_Import Gwen KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="20">
+        <f>IFERROR('_Import Gwen KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="20">
+        <f>IFERROR('_Import Gwen KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="19">
+        <f>IFERROR('_Import Miko KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B13" s="19">
+        <f>IFERROR('_Import Miko KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="19">
+        <f>IFERROR('_Import Miko KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="20">
+        <f>IFERROR('_Import Miko KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="20">
+        <f>IFERROR('_Import Miko KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="20">
+        <f>IFERROR('_Import Miko KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="20">
+        <f>IFERROR('_Import Miko KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="19">
+        <f>IFERROR('_Import Concept KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B14" s="19">
+        <f>IFERROR('_Import Concept KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="19">
+        <f>IFERROR('_Import Concept KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="20">
+        <f>IFERROR('_Import Concept KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="20">
+        <f>IFERROR('_Import Concept KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="20">
+        <f>IFERROR('_Import Concept KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="20">
+        <f>IFERROR('_Import Concept KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="19">
+        <f>IFERROR('_Import Daily KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B15" s="19">
+        <f>IFERROR('_Import Daily KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="19">
+        <f>IFERROR('_Import Daily KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>IFERROR('_Import Daily KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="20">
+        <f>IFERROR('_Import Daily KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="20">
+        <f>IFERROR('_Import Daily KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="20">
+        <f>IFERROR('_Import Daily KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="19">
+        <f>IFERROR('_Import Prime KPI'!A1,"")</f>
+        <v/>
+      </c>
+      <c r="B16" s="19">
+        <f>IFERROR('_Import Prime KPI'!B1,"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="19">
+        <f>IFERROR('_Import Prime KPI'!C1,"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>IFERROR('_Import Prime KPI'!D1,"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="20">
+        <f>IFERROR('_Import Prime KPI'!E1,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="20">
+        <f>IFERROR('_Import Prime KPI'!F1,"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="20">
+        <f>IFERROR('_Import Prime KPI'!G1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="19">
         <f>IFERROR('_Import Yuri KPI'!A1,"")</f>
         <v/>
       </c>
-      <c r="B5" s="19">
+      <c r="B17" s="19">
         <f>IFERROR('_Import Yuri KPI'!B1,"")</f>
         <v/>
       </c>
-      <c r="C5" s="19">
+      <c r="C17" s="19">
         <f>IFERROR('_Import Yuri KPI'!C1,"")</f>
         <v/>
       </c>
-      <c r="D5" s="20">
+      <c r="D17" s="20">
         <f>IFERROR('_Import Yuri KPI'!D1,"")</f>
         <v/>
       </c>
-      <c r="E5" s="20">
+      <c r="E17" s="20">
         <f>IFERROR('_Import Yuri KPI'!E1,"")</f>
         <v/>
       </c>
-      <c r="F5" s="20">
+      <c r="F17" s="20">
         <f>IFERROR('_Import Yuri KPI'!F1,"")</f>
         <v/>
       </c>
-      <c r="G5" s="20">
+      <c r="G17" s="20">
         <f>IFERROR('_Import Yuri KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="19">
-        <f>IFERROR('_Import Tuna KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B6" s="19">
-        <f>IFERROR('_Import Tuna KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C6" s="19">
-        <f>IFERROR('_Import Tuna KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D6" s="20">
-        <f>IFERROR('_Import Tuna KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E6" s="20">
-        <f>IFERROR('_Import Tuna KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F6" s="20">
-        <f>IFERROR('_Import Tuna KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G6" s="20">
-        <f>IFERROR('_Import Tuna KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="19">
-        <f>IFERROR('_Import Plat KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B7" s="19">
-        <f>IFERROR('_Import Plat KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C7" s="19">
-        <f>IFERROR('_Import Plat KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D7" s="20">
-        <f>IFERROR('_Import Plat KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E7" s="20">
-        <f>IFERROR('_Import Plat KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="20">
-        <f>IFERROR('_Import Plat KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="20">
-        <f>IFERROR('_Import Plat KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="19">
-        <f>IFERROR('_Import Chella KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B8" s="19">
-        <f>IFERROR('_Import Chella KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C8" s="19">
-        <f>IFERROR('_Import Chella KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="20">
-        <f>IFERROR('_Import Chella KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E8" s="20">
-        <f>IFERROR('_Import Chella KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="20">
-        <f>IFERROR('_Import Chella KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G8" s="20">
-        <f>IFERROR('_Import Chella KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="19">
-        <f>IFERROR('_Import Moneyheist KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B9" s="19">
-        <f>IFERROR('_Import Moneyheist KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C9" s="19">
-        <f>IFERROR('_Import Moneyheist KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D9" s="20">
-        <f>IFERROR('_Import Moneyheist KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E9" s="20">
-        <f>IFERROR('_Import Moneyheist KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F9" s="20">
-        <f>IFERROR('_Import Moneyheist KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G9" s="20">
-        <f>IFERROR('_Import Moneyheist KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="19">
-        <f>IFERROR('_Import Seb KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B10" s="19">
-        <f>IFERROR('_Import Seb KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C10" s="19">
-        <f>IFERROR('_Import Seb KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D10" s="20">
-        <f>IFERROR('_Import Seb KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E10" s="20">
-        <f>IFERROR('_Import Seb KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F10" s="20">
-        <f>IFERROR('_Import Seb KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G10" s="20">
-        <f>IFERROR('_Import Seb KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="19">
-        <f>IFERROR('_Import Pricey KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B11" s="19">
-        <f>IFERROR('_Import Pricey KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C11" s="19">
-        <f>IFERROR('_Import Pricey KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D11" s="20">
-        <f>IFERROR('_Import Pricey KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E11" s="20">
-        <f>IFERROR('_Import Pricey KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="20">
-        <f>IFERROR('_Import Pricey KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G11" s="20">
-        <f>IFERROR('_Import Pricey KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="19">
-        <f>IFERROR('_Import Seanok KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B12" s="19">
-        <f>IFERROR('_Import Seanok KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C12" s="19">
-        <f>IFERROR('_Import Seanok KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="20">
-        <f>IFERROR('_Import Seanok KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E12" s="20">
-        <f>IFERROR('_Import Seanok KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="20">
-        <f>IFERROR('_Import Seanok KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G12" s="20">
-        <f>IFERROR('_Import Seanok KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="19">
-        <f>IFERROR('_Import Gwen KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B13" s="19">
-        <f>IFERROR('_Import Gwen KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C13" s="19">
-        <f>IFERROR('_Import Gwen KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="20">
-        <f>IFERROR('_Import Gwen KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E13" s="20">
-        <f>IFERROR('_Import Gwen KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F13" s="20">
-        <f>IFERROR('_Import Gwen KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G13" s="20">
-        <f>IFERROR('_Import Gwen KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="19">
-        <f>IFERROR('_Import Miko KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B14" s="19">
-        <f>IFERROR('_Import Miko KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C14" s="19">
-        <f>IFERROR('_Import Miko KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D14" s="20">
-        <f>IFERROR('_Import Miko KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E14" s="20">
-        <f>IFERROR('_Import Miko KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="20">
-        <f>IFERROR('_Import Miko KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G14" s="20">
-        <f>IFERROR('_Import Miko KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="19">
-        <f>IFERROR('_Import Concept KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B15" s="19">
-        <f>IFERROR('_Import Concept KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C15" s="19">
-        <f>IFERROR('_Import Concept KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D15" s="20">
-        <f>IFERROR('_Import Concept KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E15" s="20">
-        <f>IFERROR('_Import Concept KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="20">
-        <f>IFERROR('_Import Concept KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G15" s="20">
-        <f>IFERROR('_Import Concept KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="19">
-        <f>IFERROR('_Import Daily KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B16" s="19">
-        <f>IFERROR('_Import Daily KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C16" s="19">
-        <f>IFERROR('_Import Daily KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="20">
-        <f>IFERROR('_Import Daily KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E16" s="20">
-        <f>IFERROR('_Import Daily KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="20">
-        <f>IFERROR('_Import Daily KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G16" s="20">
-        <f>IFERROR('_Import Daily KPI'!G1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="19">
-        <f>IFERROR('_Import Prime KPI'!A1,"")</f>
-        <v/>
-      </c>
-      <c r="B17" s="19">
-        <f>IFERROR('_Import Prime KPI'!B1,"")</f>
-        <v/>
-      </c>
-      <c r="C17" s="19">
-        <f>IFERROR('_Import Prime KPI'!C1,"")</f>
-        <v/>
-      </c>
-      <c r="D17" s="20">
-        <f>IFERROR('_Import Prime KPI'!D1,"")</f>
-        <v/>
-      </c>
-      <c r="E17" s="20">
-        <f>IFERROR('_Import Prime KPI'!E1,"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="20">
-        <f>IFERROR('_Import Prime KPI'!F1,"")</f>
-        <v/>
-      </c>
-      <c r="G17" s="20">
-        <f>IFERROR('_Import Prime KPI'!G1,"")</f>
         <v/>
       </c>
     </row>
@@ -53325,7 +53325,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>{IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!B4:B203"),IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!AC4:AC203"),IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!W4:W203"),IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - Book'!AA4:AA203")}</f>
+        <f>{IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!B4:B203"),IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!AC4:AC203"),IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!W4:W203"),IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!AA4:AA203")}</f>
         <v/>
       </c>
     </row>
@@ -53345,7 +53345,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Prime - FTD List'!A5:E204")</f>
+        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - FTD List'!A5:E204")</f>
         <v/>
       </c>
     </row>
@@ -53365,7 +53365,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1aWOmLGt-ajmq4lGyc2FFA-JsJqrIBogv0Cj0NKE2gKQ", "'Team &amp; KPI Targets'!A5:G5")</f>
+        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Team &amp; KPI Targets'!A5:G5")</f>
         <v/>
       </c>
     </row>
@@ -53385,7 +53385,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Book'!A4:O203")</f>
+        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Book'!A4:O203")</f>
         <v/>
       </c>
     </row>
@@ -53405,7 +53405,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE("1_MRriw8lIFqUf6393GbCnTyzLwpAeLRmkIVhT6BQUZ8", "'Yuri - Activity Log'!A5:E5004")</f>
+        <f>IMPORTRANGE("1E2DMtbb0qnQMj6PLoA3xPq59m3Gt0vnJl7UopBaMqhc", "'Tuna - Activity Log'!A5:E5004")</f>
         <v/>
       </c>
     </row>

</xml_diff>